<commit_message>
Δημοσίευση: Microsoft Defender for Cloud Apps (Defender Up Close, μέρος 4)
- Πέντε εικόνες από το tenant και διορθώσεις διαδρομών στο Defender portal
  (Advanced features, App governance → Entra ID, ονόματα anomaly policies)
- Αντιστοίχιση σε ΚΥΑ 1689/2025, NIS2, ISO 27001 και GDPR, με τα τέσσερα xlsx
- Links προς τη Βιβλιοθήκη KQL (oauth-consent, mass-download)
- Link «Νέο στη σειρά» στα MDE, MDO, MDI με if-published
- Popup αρχικής (STORAGE_KEY 23) και homeHighlight

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011CBWyyzeZ3YgfEffDRgT4h
</commit_message>
<xml_diff>
--- a/static/downloads/gdpr-2016-679-microsoft-365-checklist.xlsx
+++ b/static/downloads/gdpr-2016-679-microsoft-365-checklist.xlsx
@@ -2030,7 +2030,11 @@
           <t>A.5.19, A.5.21, A.5.23</t>
         </is>
       </c>
-      <c r="M18" s="7" t="n"/>
+      <c r="M18" s="7" t="inlineStr">
+        <is>
+          <t>https://thecybersec.gr/posts/microsoft-defender-up-close-series/microsoft-defender-for-cloud-apps-deep-dive/</t>
+        </is>
+      </c>
       <c r="N18" s="8" t="n"/>
       <c r="O18" s="8" t="n"/>
       <c r="P18" s="8" t="n"/>
@@ -3230,7 +3234,11 @@
           <t>A.5.14, A.5.23</t>
         </is>
       </c>
-      <c r="M36" s="7" t="n"/>
+      <c r="M36" s="7" t="inlineStr">
+        <is>
+          <t>https://thecybersec.gr/posts/microsoft-defender-up-close-series/microsoft-defender-for-cloud-apps-deep-dive/</t>
+        </is>
+      </c>
       <c r="N36" s="8" t="n"/>
       <c r="O36" s="8" t="n"/>
       <c r="P36" s="8" t="n"/>

</xml_diff>